<commit_message>
t - Commented GitLatch Commit @ 2024-7-2-11-9-27-460
</commit_message>
<xml_diff>
--- a/Test Table.xlsx
+++ b/Test Table.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27827"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{84E8E7B6-93B4-AC4F-A130-3D6DE145B92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F03D917-DB69-4FCF-B949-0393B1BCEB96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="12440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -76,7 +76,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -448,12 +448,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="E3:K13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="5" max="8" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="5:11">
       <c r="E3" t="s">
         <v>0</v>
       </c>
@@ -470,7 +470,7 @@
         <v>1111</v>
       </c>
     </row>
-    <row r="4" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="5:11">
       <c r="E4" t="s">
         <v>4</v>
       </c>
@@ -484,7 +484,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="5" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="5:11">
       <c r="E5" t="s">
         <v>5</v>
       </c>
@@ -498,7 +498,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="6" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="5:11">
       <c r="E6" t="s">
         <v>6</v>
       </c>
@@ -512,7 +512,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="7" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="5:11">
       <c r="E7" t="s">
         <v>7</v>
       </c>
@@ -526,7 +526,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="8" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="5:11">
       <c r="E8" t="s">
         <v>8</v>
       </c>
@@ -537,7 +537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="5:11">
       <c r="E9" t="s">
         <v>9</v>
       </c>
@@ -551,7 +551,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="10" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="5:11">
       <c r="E10" t="s">
         <v>10</v>
       </c>
@@ -565,7 +565,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="11" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="5:11">
       <c r="E11" t="s">
         <v>11</v>
       </c>
@@ -579,7 +579,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="12" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="5:11">
       <c r="E12" t="s">
         <v>9</v>
       </c>
@@ -593,7 +593,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="5:11">
       <c r="E13" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
Test.xlsx - Commented GitLatch Commit @ 2024-7-2-16-57-51-399
</commit_message>
<xml_diff>
--- a/Test Table.xlsx
+++ b/Test Table.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10311"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{67355502-81B1-4C35-AA00-BAC146792987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{584DF1DD-1E16-5649-ABD4-02B4080F1F54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="12440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -76,7 +76,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -448,12 +448,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="E3:K13"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="8" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="5:11">
+    <row r="3" spans="5:11" x14ac:dyDescent="0.2">
       <c r="E3" t="s">
         <v>0</v>
       </c>
@@ -470,7 +470,7 @@
         <v>1111</v>
       </c>
     </row>
-    <row r="4" spans="5:11">
+    <row r="4" spans="5:11" x14ac:dyDescent="0.2">
       <c r="E4" t="s">
         <v>4</v>
       </c>
@@ -484,7 +484,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="5" spans="5:11">
+    <row r="5" spans="5:11" x14ac:dyDescent="0.2">
       <c r="E5" t="s">
         <v>5</v>
       </c>
@@ -498,7 +498,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="6" spans="5:11">
+    <row r="6" spans="5:11" x14ac:dyDescent="0.2">
       <c r="E6" t="s">
         <v>6</v>
       </c>
@@ -512,7 +512,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="7" spans="5:11">
+    <row r="7" spans="5:11" x14ac:dyDescent="0.2">
       <c r="E7" t="s">
         <v>7</v>
       </c>
@@ -526,7 +526,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="8" spans="5:11">
+    <row r="8" spans="5:11" x14ac:dyDescent="0.2">
       <c r="E8" t="s">
         <v>8</v>
       </c>
@@ -537,7 +537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="5:11">
+    <row r="9" spans="5:11" x14ac:dyDescent="0.2">
       <c r="E9" t="s">
         <v>9</v>
       </c>
@@ -551,7 +551,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="10" spans="5:11">
+    <row r="10" spans="5:11" x14ac:dyDescent="0.2">
       <c r="E10" t="s">
         <v>10</v>
       </c>
@@ -565,7 +565,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="11" spans="5:11">
+    <row r="11" spans="5:11" x14ac:dyDescent="0.2">
       <c r="E11" t="s">
         <v>11</v>
       </c>
@@ -579,7 +579,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="12" spans="5:11">
+    <row r="12" spans="5:11" x14ac:dyDescent="0.2">
       <c r="E12" t="s">
         <v>9</v>
       </c>
@@ -593,7 +593,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="5:11">
+    <row r="13" spans="5:11" x14ac:dyDescent="0.2">
       <c r="E13" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
eree.xlsx - Commented GitLatch Commit @ 2024-7-2-12-3-51-784
</commit_message>
<xml_diff>
--- a/Test Table.xlsx
+++ b/Test Table.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10311"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27827"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D84682C-26E7-C84A-9C51-6F0E8D8C5727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C46F835D-1DB0-4D99-91F6-8649C18405D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="12440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -76,7 +76,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -448,12 +448,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="E3:K13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="5" max="8" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="5:11">
       <c r="E3" t="s">
         <v>0</v>
       </c>
@@ -470,7 +470,7 @@
         <v>1111</v>
       </c>
     </row>
-    <row r="4" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="5:11">
       <c r="E4" t="s">
         <v>4</v>
       </c>
@@ -484,7 +484,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="5" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="5:11">
       <c r="E5" t="s">
         <v>5</v>
       </c>
@@ -498,7 +498,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="6" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="5:11">
       <c r="E6" t="s">
         <v>6</v>
       </c>
@@ -512,7 +512,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="7" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="5:11">
       <c r="E7" t="s">
         <v>7</v>
       </c>
@@ -526,7 +526,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="8" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="5:11">
       <c r="E8" t="s">
         <v>8</v>
       </c>
@@ -537,7 +537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="5:11">
       <c r="E9" t="s">
         <v>9</v>
       </c>
@@ -551,7 +551,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="10" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="5:11">
       <c r="E10" t="s">
         <v>10</v>
       </c>
@@ -565,7 +565,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="11" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="5:11">
       <c r="E11" t="s">
         <v>11</v>
       </c>
@@ -579,7 +579,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="12" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="5:11">
       <c r="E12" t="s">
         <v>9</v>
       </c>
@@ -593,7 +593,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="5:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="5:11">
       <c r="E13" t="s">
         <v>12</v>
       </c>
@@ -609,7 +609,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>